<commit_message>
Updated guaranteed dispatch specifically for fuel oil plants, which are running in some parts of Mexico where there is no access to gas infrastructure, like Baja Sur.
</commit_message>
<xml_diff>
--- a/InputData/elec/BGDPbES/BAU Guaranteed Dispatch Perc by Elec Source.xlsx
+++ b/InputData/elec/BGDPbES/BAU Guaranteed Dispatch Perc by Elec Source.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RobbieOrvis\Models\Mexico\Models\eps-mexico\InputData\elec\BGDPbES\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63713A03-AA73-45DF-8CCC-9E1B77428528}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{573220F2-9BB9-405B-ABE6-C6D0A46C669A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{80F9C2E1-CAFD-42D4-BC6F-A67AD09DB17B}"/>
   </bookViews>
@@ -3591,154 +3591,154 @@
         <v>46</v>
       </c>
       <c r="B17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AC17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AD17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AJ17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AK17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AL17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AM17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AN17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AO17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AP17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AQ17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AR17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AT17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AV17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AW17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AX17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AY17">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18" spans="1:51">
@@ -5132,18 +5132,18 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -5165,18 +5165,18 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{28F56A48-4057-4FCF-82D0-97D2AB650057}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E3AE0EBA-E7D6-42C9-A9CD-15E21C9A6DFC}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{28F56A48-4057-4FCF-82D0-97D2AB650057}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>